<commit_message>
Store image through cloudinary
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,6 +31,10 @@
       <color theme="10"/>
       <sz val="12"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <color rgb="000000FF"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="2">
@@ -54,9 +58,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -607,6 +612,141 @@
       <c r="D7" t="inlineStr">
         <is>
           <t>11:18:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Shubhangi Sudhakar Ingle</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Cubeage AI ML</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>16:05:01</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Upload failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Shubhangi Sudhakar Ingle</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Cubeage AI ML</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>16:42:52</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Upload failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Shubhangi Sudhakar Ingle</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Cubeage Full Stack Internship</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>16:49:49</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/do2oynvcf/image/upload/v1785928797/Shubhangi_Sudhakar_Ingle_Cubeage%20Full%20Stack%20Internship_20260805_164949.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Shubhangi Sudhakar Ingle</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cubeage Full Stack Internship</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>16:54:16</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/do2oynvcf/image/upload/v1785929062/Shubhangi_Sudhakar_Ingle_Cubeage%20Full%20Stack%20Internship_20260805_165416.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Shubhangi Sudhakar Ingle</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Cubeage AI ML</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>16:59:48</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>View Photo</t>
         </is>
       </c>
     </row>
@@ -617,6 +757,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Create different sheet for different subject
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -745,6 +745,114 @@
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>View Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Shubhangi Sudhakar Ingle</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Cubeage Full Stack Internship</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>17:24:40</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>View Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Shubhangi Sudhakar Ingle</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Cubeage Full Stack Internship</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>17:27:40</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>View Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Shubhangi Sudhakar Ingle</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Cubeage AI ML</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>17:28:39</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>View Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Shreya Jangam</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Cubeage AI ML</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>17:29:51</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>View Photo</t>
         </is>
@@ -760,6 +868,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>